<commit_message>
refactor: benchmark with logarithm
</commit_message>
<xml_diff>
--- a/4a/bst_benchmark.xlsx
+++ b/4a/bst_benchmark.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\tr3sl9\2_sem\4a\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{26837345-AF42-44E2-B8F6-10E5660B5BDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4893B824-3641-454F-BAED-7B4A483F13C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{819852D7-CD4B-4096-9E24-0C73342B040C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{ED679D53-E4ED-41AE-BC7A-34F45A594A49}"/>
   </bookViews>
   <sheets>
     <sheet name="bst_benchmark" sheetId="1" r:id="rId1"/>
@@ -628,7 +628,11 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>Benchmark BST</a:t>
+              <a:t>BST</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" baseline="0"/>
+              <a:t> benchmark</a:t>
             </a:r>
             <a:endParaRPr lang="ru-RU"/>
           </a:p>
@@ -671,7 +675,7 @@
         <c:varyColors val="0"/>
         <c:ser>
           <c:idx val="1"/>
-          <c:order val="1"/>
+          <c:order val="0"/>
           <c:tx>
             <c:strRef>
               <c:f>bst_benchmark!$B$1</c:f>
@@ -697,198 +701,318 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>bst_benchmark!$A$2:$A$31</c:f>
+              <c:f>bst_benchmark!$A$2:$A$51</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="30"/>
+                <c:ptCount val="50"/>
                 <c:pt idx="0">
-                  <c:v>40000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>80000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>120000</c:v>
+                  <c:v>300000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>160000</c:v>
+                  <c:v>400000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>200000</c:v>
+                  <c:v>500000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>240000</c:v>
+                  <c:v>600000</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>280000</c:v>
+                  <c:v>700000</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>320000</c:v>
+                  <c:v>800000</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>360000</c:v>
+                  <c:v>900000</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>400000</c:v>
+                  <c:v>1000000</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>440000</c:v>
+                  <c:v>1100000</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>480000</c:v>
+                  <c:v>1200000</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>520000</c:v>
+                  <c:v>1300000</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>560000</c:v>
+                  <c:v>1400000</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>600000</c:v>
+                  <c:v>1500000</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>640000</c:v>
+                  <c:v>1600000</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>680000</c:v>
+                  <c:v>1700000</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>720000</c:v>
+                  <c:v>1800000</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>760000</c:v>
+                  <c:v>1900000</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>800000</c:v>
+                  <c:v>2000000</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>840000</c:v>
+                  <c:v>2100000</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>880000</c:v>
+                  <c:v>2200000</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>920000</c:v>
+                  <c:v>2300000</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>960000</c:v>
+                  <c:v>2400000</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>1000000</c:v>
+                  <c:v>2500000</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>1040000</c:v>
+                  <c:v>2600000</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>1080000</c:v>
+                  <c:v>2700000</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>1120000</c:v>
+                  <c:v>2800000</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>1160000</c:v>
+                  <c:v>2900000</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>1200000</c:v>
+                  <c:v>3000000</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>3100000</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>3200000</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>3300000</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>3400000</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>3500000</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>3600000</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>3700000</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>3800000</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>3900000</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>4000000</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>4100000</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>4200000</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>4300000</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>4400000</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>4500000</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>4600000</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>4700000</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>4800000</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>4900000</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>5000000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>bst_benchmark!$B$2:$B$31</c:f>
+              <c:f>bst_benchmark!$B$2:$B$51</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="30"/>
+                <c:ptCount val="50"/>
                 <c:pt idx="0">
-                  <c:v>17343248</c:v>
+                  <c:v>1358121.25</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>18401416.5</c:v>
+                  <c:v>1498855.85</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>18414816.050000001</c:v>
+                  <c:v>1613086.5</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>19237056.699999999</c:v>
+                  <c:v>1653464.65</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>19840616.199999999</c:v>
+                  <c:v>1760770.75</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>20735293.800000001</c:v>
+                  <c:v>1794289.45</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>20917200.399999999</c:v>
+                  <c:v>1808732.85</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>21616176.300000001</c:v>
+                  <c:v>1848449.05</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>21618384.399999999</c:v>
+                  <c:v>1924946.4</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>22060551.699999999</c:v>
+                  <c:v>1974841.15</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>22077960.449999999</c:v>
+                  <c:v>2142021.2000000002</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>22851930.949999999</c:v>
+                  <c:v>2027145.95</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>22951123.800000001</c:v>
+                  <c:v>2023527.3</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>23359211.399999999</c:v>
+                  <c:v>2078076.85</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>23264916.75</c:v>
+                  <c:v>2035593.05</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>23738586.449999999</c:v>
+                  <c:v>2084409.15</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>23709823.800000001</c:v>
+                  <c:v>2061872.85</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>24133547.350000001</c:v>
+                  <c:v>2081575.25</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>24096246.050000001</c:v>
+                  <c:v>2107733.2000000002</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>24643209.149999999</c:v>
+                  <c:v>2127574.65</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>24475778.899999999</c:v>
+                  <c:v>2137816.2000000002</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>24755635.800000001</c:v>
+                  <c:v>2209449.5499999998</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>24762640.699999999</c:v>
+                  <c:v>2164490.2000000002</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>25119014.300000001</c:v>
+                  <c:v>2199083.5</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>25435974.800000001</c:v>
+                  <c:v>2192899.5499999998</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>25315170.949999999</c:v>
+                  <c:v>2218219.4</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>25760840.699999999</c:v>
+                  <c:v>2423310.9500000002</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>25520049.75</c:v>
+                  <c:v>2236843.6</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>26055262.600000001</c:v>
+                  <c:v>2235982.4500000002</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>25990273.350000001</c:v>
+                  <c:v>2247601.25</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>2248765.5499999998</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>2506534.7999999998</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>2278272.25</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>2351233.15</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>2327192.4500000002</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>2334283.35</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>2477672.1</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>2355185.4</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>2367498.65</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>2398683.0499999998</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>2392995.7000000002</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>2506931.2000000002</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>2506721.35</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>2441812.15</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>2444845.5499999998</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>2448101.85</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>2476419</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>2478129</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>2498015.2000000002</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>2525736.6</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -896,13 +1020,13 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-4164-4F07-83C9-B83DC0396D4C}"/>
+              <c16:uniqueId val="{00000001-D90E-4B35-9A47-5D27D3294680}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="2"/>
-          <c:order val="2"/>
+          <c:order val="1"/>
           <c:tx>
             <c:strRef>
               <c:f>bst_benchmark!$C$1</c:f>
@@ -928,198 +1052,318 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>bst_benchmark!$A$2:$A$31</c:f>
+              <c:f>bst_benchmark!$A$2:$A$51</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="30"/>
+                <c:ptCount val="50"/>
                 <c:pt idx="0">
-                  <c:v>40000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>80000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>120000</c:v>
+                  <c:v>300000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>160000</c:v>
+                  <c:v>400000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>200000</c:v>
+                  <c:v>500000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>240000</c:v>
+                  <c:v>600000</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>280000</c:v>
+                  <c:v>700000</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>320000</c:v>
+                  <c:v>800000</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>360000</c:v>
+                  <c:v>900000</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>400000</c:v>
+                  <c:v>1000000</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>440000</c:v>
+                  <c:v>1100000</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>480000</c:v>
+                  <c:v>1200000</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>520000</c:v>
+                  <c:v>1300000</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>560000</c:v>
+                  <c:v>1400000</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>600000</c:v>
+                  <c:v>1500000</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>640000</c:v>
+                  <c:v>1600000</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>680000</c:v>
+                  <c:v>1700000</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>720000</c:v>
+                  <c:v>1800000</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>760000</c:v>
+                  <c:v>1900000</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>800000</c:v>
+                  <c:v>2000000</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>840000</c:v>
+                  <c:v>2100000</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>880000</c:v>
+                  <c:v>2200000</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>920000</c:v>
+                  <c:v>2300000</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>960000</c:v>
+                  <c:v>2400000</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>1000000</c:v>
+                  <c:v>2500000</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>1040000</c:v>
+                  <c:v>2600000</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>1080000</c:v>
+                  <c:v>2700000</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>1120000</c:v>
+                  <c:v>2800000</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>1160000</c:v>
+                  <c:v>2900000</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>1200000</c:v>
+                  <c:v>3000000</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>3100000</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>3200000</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>3300000</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>3400000</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>3500000</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>3600000</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>3700000</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>3800000</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>3900000</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>4000000</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>4100000</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>4200000</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>4300000</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>4400000</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>4500000</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>4600000</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>4700000</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>4800000</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>4900000</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>5000000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>bst_benchmark!$C$2:$C$31</c:f>
+              <c:f>bst_benchmark!$C$2:$C$51</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="30"/>
+                <c:ptCount val="50"/>
                 <c:pt idx="0">
-                  <c:v>6805596.2000000002</c:v>
+                  <c:v>635573.85</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>7394723.75</c:v>
+                  <c:v>727713.2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>7949136.4500000002</c:v>
+                  <c:v>815957.85</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>8762055.8499999996</c:v>
+                  <c:v>893278.6</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>8797128.4000000004</c:v>
+                  <c:v>938273.65</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>9214856.75</c:v>
+                  <c:v>969891.9</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>9675506.5500000007</c:v>
+                  <c:v>1004344.9</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>10115129.1</c:v>
+                  <c:v>1072336.6499999999</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>10065218.15</c:v>
+                  <c:v>1047533.05</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>10224644.75</c:v>
+                  <c:v>1075121.45</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>10135115.449999999</c:v>
+                  <c:v>1147452.3999999999</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>10956676.65</c:v>
+                  <c:v>1125534.95</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>10974587.5</c:v>
+                  <c:v>1214483.3</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>11281438.199999999</c:v>
+                  <c:v>1158069.95</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>11378255.65</c:v>
+                  <c:v>1237375.75</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>11681059.1</c:v>
+                  <c:v>1199976.8</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>11482081.5</c:v>
+                  <c:v>1206945.2</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>11921759.75</c:v>
+                  <c:v>1200658.6000000001</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>11919652.550000001</c:v>
+                  <c:v>1217585.05</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>12246073.85</c:v>
+                  <c:v>1225443</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>12311928.300000001</c:v>
+                  <c:v>1229291.6499999999</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>12589391.65</c:v>
+                  <c:v>1284765.45</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>12416321.550000001</c:v>
+                  <c:v>1254879.3999999999</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>12681250.35</c:v>
+                  <c:v>1269693.1000000001</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>12917494.85</c:v>
+                  <c:v>1272646.8999999999</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>12797113.75</c:v>
+                  <c:v>1281271.1499999999</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>12975746.199999999</c:v>
+                  <c:v>1364234.1</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>12981452</c:v>
+                  <c:v>1315081.3999999999</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>13174044.5</c:v>
+                  <c:v>1319610.6499999999</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>13201579.449999999</c:v>
+                  <c:v>1340089.45</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>1339324.3500000001</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>1402569.65</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>1349274.9</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>1395239.25</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>1430820.5</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>1378926.05</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>1453784.2</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>1399157.7</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>1455847.9</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>1487554.55</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>1405669.75</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>1441242.55</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>1424099.3</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>1512604.8</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>1445342.95</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>1449203.8</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>1462577.3</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>1461769.35</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>1486407.65</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>1472798.25</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1127,13 +1371,13 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-4164-4F07-83C9-B83DC0396D4C}"/>
+              <c16:uniqueId val="{00000002-D90E-4B35-9A47-5D27D3294680}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="3"/>
-          <c:order val="3"/>
+          <c:order val="2"/>
           <c:tx>
             <c:strRef>
               <c:f>bst_benchmark!$D$1</c:f>
@@ -1159,198 +1403,318 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>bst_benchmark!$A$2:$A$31</c:f>
+              <c:f>bst_benchmark!$A$2:$A$51</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="30"/>
+                <c:ptCount val="50"/>
                 <c:pt idx="0">
-                  <c:v>40000</c:v>
+                  <c:v>100000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>80000</c:v>
+                  <c:v>200000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>120000</c:v>
+                  <c:v>300000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>160000</c:v>
+                  <c:v>400000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>200000</c:v>
+                  <c:v>500000</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>240000</c:v>
+                  <c:v>600000</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>280000</c:v>
+                  <c:v>700000</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>320000</c:v>
+                  <c:v>800000</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>360000</c:v>
+                  <c:v>900000</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>400000</c:v>
+                  <c:v>1000000</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>440000</c:v>
+                  <c:v>1100000</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>480000</c:v>
+                  <c:v>1200000</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>520000</c:v>
+                  <c:v>1300000</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>560000</c:v>
+                  <c:v>1400000</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>600000</c:v>
+                  <c:v>1500000</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>640000</c:v>
+                  <c:v>1600000</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>680000</c:v>
+                  <c:v>1700000</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>720000</c:v>
+                  <c:v>1800000</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>760000</c:v>
+                  <c:v>1900000</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>800000</c:v>
+                  <c:v>2000000</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>840000</c:v>
+                  <c:v>2100000</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>880000</c:v>
+                  <c:v>2200000</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>920000</c:v>
+                  <c:v>2300000</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>960000</c:v>
+                  <c:v>2400000</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>1000000</c:v>
+                  <c:v>2500000</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>1040000</c:v>
+                  <c:v>2600000</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>1080000</c:v>
+                  <c:v>2700000</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>1120000</c:v>
+                  <c:v>2800000</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>1160000</c:v>
+                  <c:v>2900000</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>1200000</c:v>
+                  <c:v>3000000</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>3100000</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>3200000</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>3300000</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>3400000</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>3500000</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>3600000</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>3700000</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>3800000</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>3900000</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>4000000</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>4100000</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>4200000</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>4300000</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>4400000</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>4500000</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>4600000</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>4700000</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>4800000</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>4900000</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>5000000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>bst_benchmark!$D$2:$D$31</c:f>
+              <c:f>bst_benchmark!$D$2:$D$51</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="30"/>
+                <c:ptCount val="50"/>
                 <c:pt idx="0">
-                  <c:v>13100014.800000001</c:v>
+                  <c:v>1460569</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>13642298.449999999</c:v>
+                  <c:v>1547751.25</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>14445127.949999999</c:v>
+                  <c:v>1578130.95</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>15100082.1</c:v>
+                  <c:v>1664300.4</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>15220334.75</c:v>
+                  <c:v>1735589.75</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>15697415.85</c:v>
+                  <c:v>1736427.8</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>15909116.4</c:v>
+                  <c:v>1759948.55</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>16433472.550000001</c:v>
+                  <c:v>1832080.05</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>16545615.25</c:v>
+                  <c:v>1898698.35</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>17387639.100000001</c:v>
+                  <c:v>1920249.95</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>16654382.85</c:v>
+                  <c:v>1920279.95</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>17707149.850000001</c:v>
+                  <c:v>1967068.2</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>17772744.399999999</c:v>
+                  <c:v>1931633.95</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>18381445.149999999</c:v>
+                  <c:v>1951131.2</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>18160294.300000001</c:v>
+                  <c:v>1997880.05</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>18608343.199999999</c:v>
+                  <c:v>2108976</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>18537034.050000001</c:v>
+                  <c:v>2022208.3</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>18887193.100000001</c:v>
+                  <c:v>2092111.35</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>19051849</c:v>
+                  <c:v>2032602.55</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>19044358.5</c:v>
+                  <c:v>2038386.3</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>19212787.25</c:v>
+                  <c:v>2055079.3</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>19642815.850000001</c:v>
+                  <c:v>2102368.0499999998</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>19300379</c:v>
+                  <c:v>2084135.95</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>19739062.600000001</c:v>
+                  <c:v>2091744.6</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>20010225.600000001</c:v>
+                  <c:v>2092069.85</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>19771113.449999999</c:v>
+                  <c:v>2090982</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>20098544.350000001</c:v>
+                  <c:v>2219170.2999999998</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>20213931.649999999</c:v>
+                  <c:v>2127354.25</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>20531292.25</c:v>
+                  <c:v>2118675.9</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>20529016</c:v>
+                  <c:v>2126855.4500000002</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>2129893.0499999998</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>2298258.5</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>2206322.7999999998</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>2224627.1</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>2162826.35</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>2224406.9</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>2311302.75</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>2183803.5499999998</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>2191922.2000000002</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>2219953.4500000002</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>2188174.4</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>2222342.5499999998</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>2244952</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>2255852.2999999998</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>2324724.75</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>2262398.85</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>2264053.25</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>2261888.4</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>2282574.4500000002</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>2282040.9</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1358,7 +1722,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-4164-4F07-83C9-B83DC0396D4C}"/>
+              <c16:uniqueId val="{00000003-D90E-4B35-9A47-5D27D3294680}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1371,266 +1735,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:smooth val="0"/>
-        <c:axId val="611531792"/>
-        <c:axId val="611534672"/>
-        <c:extLst>
-          <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-            <c15:filteredLineSeries>
-              <c15:ser>
-                <c:idx val="0"/>
-                <c:order val="0"/>
-                <c:tx>
-                  <c:strRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>bst_benchmark!$A$1</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:strCache>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>TreeSize</c:v>
-                      </c:pt>
-                    </c:strCache>
-                  </c:strRef>
-                </c:tx>
-                <c:spPr>
-                  <a:ln w="28575" cap="rnd">
-                    <a:solidFill>
-                      <a:schemeClr val="accent1"/>
-                    </a:solidFill>
-                    <a:round/>
-                  </a:ln>
-                  <a:effectLst/>
-                </c:spPr>
-                <c:marker>
-                  <c:symbol val="none"/>
-                </c:marker>
-                <c:cat>
-                  <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>bst_benchmark!$A$2:$A$31</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="30"/>
-                      <c:pt idx="0">
-                        <c:v>40000</c:v>
-                      </c:pt>
-                      <c:pt idx="1">
-                        <c:v>80000</c:v>
-                      </c:pt>
-                      <c:pt idx="2">
-                        <c:v>120000</c:v>
-                      </c:pt>
-                      <c:pt idx="3">
-                        <c:v>160000</c:v>
-                      </c:pt>
-                      <c:pt idx="4">
-                        <c:v>200000</c:v>
-                      </c:pt>
-                      <c:pt idx="5">
-                        <c:v>240000</c:v>
-                      </c:pt>
-                      <c:pt idx="6">
-                        <c:v>280000</c:v>
-                      </c:pt>
-                      <c:pt idx="7">
-                        <c:v>320000</c:v>
-                      </c:pt>
-                      <c:pt idx="8">
-                        <c:v>360000</c:v>
-                      </c:pt>
-                      <c:pt idx="9">
-                        <c:v>400000</c:v>
-                      </c:pt>
-                      <c:pt idx="10">
-                        <c:v>440000</c:v>
-                      </c:pt>
-                      <c:pt idx="11">
-                        <c:v>480000</c:v>
-                      </c:pt>
-                      <c:pt idx="12">
-                        <c:v>520000</c:v>
-                      </c:pt>
-                      <c:pt idx="13">
-                        <c:v>560000</c:v>
-                      </c:pt>
-                      <c:pt idx="14">
-                        <c:v>600000</c:v>
-                      </c:pt>
-                      <c:pt idx="15">
-                        <c:v>640000</c:v>
-                      </c:pt>
-                      <c:pt idx="16">
-                        <c:v>680000</c:v>
-                      </c:pt>
-                      <c:pt idx="17">
-                        <c:v>720000</c:v>
-                      </c:pt>
-                      <c:pt idx="18">
-                        <c:v>760000</c:v>
-                      </c:pt>
-                      <c:pt idx="19">
-                        <c:v>800000</c:v>
-                      </c:pt>
-                      <c:pt idx="20">
-                        <c:v>840000</c:v>
-                      </c:pt>
-                      <c:pt idx="21">
-                        <c:v>880000</c:v>
-                      </c:pt>
-                      <c:pt idx="22">
-                        <c:v>920000</c:v>
-                      </c:pt>
-                      <c:pt idx="23">
-                        <c:v>960000</c:v>
-                      </c:pt>
-                      <c:pt idx="24">
-                        <c:v>1000000</c:v>
-                      </c:pt>
-                      <c:pt idx="25">
-                        <c:v>1040000</c:v>
-                      </c:pt>
-                      <c:pt idx="26">
-                        <c:v>1080000</c:v>
-                      </c:pt>
-                      <c:pt idx="27">
-                        <c:v>1120000</c:v>
-                      </c:pt>
-                      <c:pt idx="28">
-                        <c:v>1160000</c:v>
-                      </c:pt>
-                      <c:pt idx="29">
-                        <c:v>1200000</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:cat>
-                <c:val>
-                  <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>bst_benchmark!$A$2:$A$31</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="30"/>
-                      <c:pt idx="0">
-                        <c:v>40000</c:v>
-                      </c:pt>
-                      <c:pt idx="1">
-                        <c:v>80000</c:v>
-                      </c:pt>
-                      <c:pt idx="2">
-                        <c:v>120000</c:v>
-                      </c:pt>
-                      <c:pt idx="3">
-                        <c:v>160000</c:v>
-                      </c:pt>
-                      <c:pt idx="4">
-                        <c:v>200000</c:v>
-                      </c:pt>
-                      <c:pt idx="5">
-                        <c:v>240000</c:v>
-                      </c:pt>
-                      <c:pt idx="6">
-                        <c:v>280000</c:v>
-                      </c:pt>
-                      <c:pt idx="7">
-                        <c:v>320000</c:v>
-                      </c:pt>
-                      <c:pt idx="8">
-                        <c:v>360000</c:v>
-                      </c:pt>
-                      <c:pt idx="9">
-                        <c:v>400000</c:v>
-                      </c:pt>
-                      <c:pt idx="10">
-                        <c:v>440000</c:v>
-                      </c:pt>
-                      <c:pt idx="11">
-                        <c:v>480000</c:v>
-                      </c:pt>
-                      <c:pt idx="12">
-                        <c:v>520000</c:v>
-                      </c:pt>
-                      <c:pt idx="13">
-                        <c:v>560000</c:v>
-                      </c:pt>
-                      <c:pt idx="14">
-                        <c:v>600000</c:v>
-                      </c:pt>
-                      <c:pt idx="15">
-                        <c:v>640000</c:v>
-                      </c:pt>
-                      <c:pt idx="16">
-                        <c:v>680000</c:v>
-                      </c:pt>
-                      <c:pt idx="17">
-                        <c:v>720000</c:v>
-                      </c:pt>
-                      <c:pt idx="18">
-                        <c:v>760000</c:v>
-                      </c:pt>
-                      <c:pt idx="19">
-                        <c:v>800000</c:v>
-                      </c:pt>
-                      <c:pt idx="20">
-                        <c:v>840000</c:v>
-                      </c:pt>
-                      <c:pt idx="21">
-                        <c:v>880000</c:v>
-                      </c:pt>
-                      <c:pt idx="22">
-                        <c:v>920000</c:v>
-                      </c:pt>
-                      <c:pt idx="23">
-                        <c:v>960000</c:v>
-                      </c:pt>
-                      <c:pt idx="24">
-                        <c:v>1000000</c:v>
-                      </c:pt>
-                      <c:pt idx="25">
-                        <c:v>1040000</c:v>
-                      </c:pt>
-                      <c:pt idx="26">
-                        <c:v>1080000</c:v>
-                      </c:pt>
-                      <c:pt idx="27">
-                        <c:v>1120000</c:v>
-                      </c:pt>
-                      <c:pt idx="28">
-                        <c:v>1160000</c:v>
-                      </c:pt>
-                      <c:pt idx="29">
-                        <c:v>1200000</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:val>
-                <c:smooth val="0"/>
-                <c:extLst>
-                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                    <c16:uniqueId val="{00000000-4164-4F07-83C9-B83DC0396D4C}"/>
-                  </c:ext>
-                </c:extLst>
-              </c15:ser>
-            </c15:filteredLineSeries>
-          </c:ext>
-        </c:extLst>
+        <c:axId val="635195624"/>
+        <c:axId val="635198864"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="611531792"/>
+        <c:axId val="635195624"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1673,7 +1782,7 @@
             <a:endParaRPr lang="ru-RU"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="611534672"/>
+        <c:crossAx val="635198864"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1681,7 +1790,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="611534672"/>
+        <c:axId val="635198864"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1732,7 +1841,7 @@
             <a:endParaRPr lang="ru-RU"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="611531792"/>
+        <c:crossAx val="635195624"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2379,23 +2488,23 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>600075</xdr:colOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>19049</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>4762</xdr:rowOff>
+      <xdr:rowOff>180975</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>600075</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>9524</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Диаграмма 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{39B0F4EF-7421-3FC1-9FB3-F58C3A528559}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FB4009CE-026F-1551-469B-787E7BBEA12D}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2712,8 +2821,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AEF029A8-3DA6-4E4B-B5E2-E62AD9F60718}">
-  <dimension ref="A1:D31"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25B5A7E0-F1F4-4E6C-A483-C61144F9EABA}">
+  <dimension ref="A1:D51"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -2732,422 +2841,702 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>40000</v>
+        <v>100000</v>
       </c>
       <c r="B2">
-        <v>17343248</v>
+        <v>1358121.25</v>
       </c>
       <c r="C2">
-        <v>6805596.2000000002</v>
+        <v>635573.85</v>
       </c>
       <c r="D2">
-        <v>13100014.800000001</v>
+        <v>1460569</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>80000</v>
+        <v>200000</v>
       </c>
       <c r="B3">
-        <v>18401416.5</v>
+        <v>1498855.85</v>
       </c>
       <c r="C3">
-        <v>7394723.75</v>
+        <v>727713.2</v>
       </c>
       <c r="D3">
-        <v>13642298.449999999</v>
+        <v>1547751.25</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>120000</v>
+        <v>300000</v>
       </c>
       <c r="B4">
-        <v>18414816.050000001</v>
+        <v>1613086.5</v>
       </c>
       <c r="C4">
-        <v>7949136.4500000002</v>
+        <v>815957.85</v>
       </c>
       <c r="D4">
-        <v>14445127.949999999</v>
+        <v>1578130.95</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>160000</v>
+        <v>400000</v>
       </c>
       <c r="B5">
-        <v>19237056.699999999</v>
+        <v>1653464.65</v>
       </c>
       <c r="C5">
-        <v>8762055.8499999996</v>
+        <v>893278.6</v>
       </c>
       <c r="D5">
-        <v>15100082.1</v>
+        <v>1664300.4</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>200000</v>
+        <v>500000</v>
       </c>
       <c r="B6">
-        <v>19840616.199999999</v>
+        <v>1760770.75</v>
       </c>
       <c r="C6">
-        <v>8797128.4000000004</v>
+        <v>938273.65</v>
       </c>
       <c r="D6">
-        <v>15220334.75</v>
+        <v>1735589.75</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7">
-        <v>240000</v>
+        <v>600000</v>
       </c>
       <c r="B7">
-        <v>20735293.800000001</v>
+        <v>1794289.45</v>
       </c>
       <c r="C7">
-        <v>9214856.75</v>
+        <v>969891.9</v>
       </c>
       <c r="D7">
-        <v>15697415.85</v>
+        <v>1736427.8</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8">
-        <v>280000</v>
+        <v>700000</v>
       </c>
       <c r="B8">
-        <v>20917200.399999999</v>
+        <v>1808732.85</v>
       </c>
       <c r="C8">
-        <v>9675506.5500000007</v>
+        <v>1004344.9</v>
       </c>
       <c r="D8">
-        <v>15909116.4</v>
+        <v>1759948.55</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9">
-        <v>320000</v>
+        <v>800000</v>
       </c>
       <c r="B9">
-        <v>21616176.300000001</v>
+        <v>1848449.05</v>
       </c>
       <c r="C9">
-        <v>10115129.1</v>
+        <v>1072336.6499999999</v>
       </c>
       <c r="D9">
-        <v>16433472.550000001</v>
+        <v>1832080.05</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10">
-        <v>360000</v>
+        <v>900000</v>
       </c>
       <c r="B10">
-        <v>21618384.399999999</v>
+        <v>1924946.4</v>
       </c>
       <c r="C10">
-        <v>10065218.15</v>
+        <v>1047533.05</v>
       </c>
       <c r="D10">
-        <v>16545615.25</v>
+        <v>1898698.35</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11">
-        <v>400000</v>
+        <v>1000000</v>
       </c>
       <c r="B11">
-        <v>22060551.699999999</v>
+        <v>1974841.15</v>
       </c>
       <c r="C11">
-        <v>10224644.75</v>
+        <v>1075121.45</v>
       </c>
       <c r="D11">
-        <v>17387639.100000001</v>
+        <v>1920249.95</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12">
-        <v>440000</v>
+        <v>1100000</v>
       </c>
       <c r="B12">
-        <v>22077960.449999999</v>
+        <v>2142021.2000000002</v>
       </c>
       <c r="C12">
-        <v>10135115.449999999</v>
+        <v>1147452.3999999999</v>
       </c>
       <c r="D12">
-        <v>16654382.85</v>
+        <v>1920279.95</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13">
-        <v>480000</v>
+        <v>1200000</v>
       </c>
       <c r="B13">
-        <v>22851930.949999999</v>
+        <v>2027145.95</v>
       </c>
       <c r="C13">
-        <v>10956676.65</v>
+        <v>1125534.95</v>
       </c>
       <c r="D13">
-        <v>17707149.850000001</v>
+        <v>1967068.2</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14">
-        <v>520000</v>
+        <v>1300000</v>
       </c>
       <c r="B14">
-        <v>22951123.800000001</v>
+        <v>2023527.3</v>
       </c>
       <c r="C14">
-        <v>10974587.5</v>
+        <v>1214483.3</v>
       </c>
       <c r="D14">
-        <v>17772744.399999999</v>
+        <v>1931633.95</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15">
-        <v>560000</v>
+        <v>1400000</v>
       </c>
       <c r="B15">
-        <v>23359211.399999999</v>
+        <v>2078076.85</v>
       </c>
       <c r="C15">
-        <v>11281438.199999999</v>
+        <v>1158069.95</v>
       </c>
       <c r="D15">
-        <v>18381445.149999999</v>
+        <v>1951131.2</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16">
-        <v>600000</v>
+        <v>1500000</v>
       </c>
       <c r="B16">
-        <v>23264916.75</v>
+        <v>2035593.05</v>
       </c>
       <c r="C16">
-        <v>11378255.65</v>
+        <v>1237375.75</v>
       </c>
       <c r="D16">
-        <v>18160294.300000001</v>
+        <v>1997880.05</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17">
-        <v>640000</v>
+        <v>1600000</v>
       </c>
       <c r="B17">
-        <v>23738586.449999999</v>
+        <v>2084409.15</v>
       </c>
       <c r="C17">
-        <v>11681059.1</v>
+        <v>1199976.8</v>
       </c>
       <c r="D17">
-        <v>18608343.199999999</v>
+        <v>2108976</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18">
-        <v>680000</v>
+        <v>1700000</v>
       </c>
       <c r="B18">
-        <v>23709823.800000001</v>
+        <v>2061872.85</v>
       </c>
       <c r="C18">
-        <v>11482081.5</v>
+        <v>1206945.2</v>
       </c>
       <c r="D18">
-        <v>18537034.050000001</v>
+        <v>2022208.3</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19">
-        <v>720000</v>
+        <v>1800000</v>
       </c>
       <c r="B19">
-        <v>24133547.350000001</v>
+        <v>2081575.25</v>
       </c>
       <c r="C19">
-        <v>11921759.75</v>
+        <v>1200658.6000000001</v>
       </c>
       <c r="D19">
-        <v>18887193.100000001</v>
+        <v>2092111.35</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20">
-        <v>760000</v>
+        <v>1900000</v>
       </c>
       <c r="B20">
-        <v>24096246.050000001</v>
+        <v>2107733.2000000002</v>
       </c>
       <c r="C20">
-        <v>11919652.550000001</v>
+        <v>1217585.05</v>
       </c>
       <c r="D20">
-        <v>19051849</v>
+        <v>2032602.55</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21">
-        <v>800000</v>
+        <v>2000000</v>
       </c>
       <c r="B21">
-        <v>24643209.149999999</v>
+        <v>2127574.65</v>
       </c>
       <c r="C21">
-        <v>12246073.85</v>
+        <v>1225443</v>
       </c>
       <c r="D21">
-        <v>19044358.5</v>
+        <v>2038386.3</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22">
-        <v>840000</v>
+        <v>2100000</v>
       </c>
       <c r="B22">
-        <v>24475778.899999999</v>
+        <v>2137816.2000000002</v>
       </c>
       <c r="C22">
-        <v>12311928.300000001</v>
+        <v>1229291.6499999999</v>
       </c>
       <c r="D22">
-        <v>19212787.25</v>
+        <v>2055079.3</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23">
-        <v>880000</v>
+        <v>2200000</v>
       </c>
       <c r="B23">
-        <v>24755635.800000001</v>
+        <v>2209449.5499999998</v>
       </c>
       <c r="C23">
-        <v>12589391.65</v>
+        <v>1284765.45</v>
       </c>
       <c r="D23">
-        <v>19642815.850000001</v>
+        <v>2102368.0499999998</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24">
-        <v>920000</v>
+        <v>2300000</v>
       </c>
       <c r="B24">
-        <v>24762640.699999999</v>
+        <v>2164490.2000000002</v>
       </c>
       <c r="C24">
-        <v>12416321.550000001</v>
+        <v>1254879.3999999999</v>
       </c>
       <c r="D24">
-        <v>19300379</v>
+        <v>2084135.95</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25">
-        <v>960000</v>
+        <v>2400000</v>
       </c>
       <c r="B25">
-        <v>25119014.300000001</v>
+        <v>2199083.5</v>
       </c>
       <c r="C25">
-        <v>12681250.35</v>
+        <v>1269693.1000000001</v>
       </c>
       <c r="D25">
-        <v>19739062.600000001</v>
+        <v>2091744.6</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26">
-        <v>1000000</v>
+        <v>2500000</v>
       </c>
       <c r="B26">
-        <v>25435974.800000001</v>
+        <v>2192899.5499999998</v>
       </c>
       <c r="C26">
-        <v>12917494.85</v>
+        <v>1272646.8999999999</v>
       </c>
       <c r="D26">
-        <v>20010225.600000001</v>
+        <v>2092069.85</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27">
-        <v>1040000</v>
+        <v>2600000</v>
       </c>
       <c r="B27">
-        <v>25315170.949999999</v>
+        <v>2218219.4</v>
       </c>
       <c r="C27">
-        <v>12797113.75</v>
+        <v>1281271.1499999999</v>
       </c>
       <c r="D27">
-        <v>19771113.449999999</v>
+        <v>2090982</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28">
-        <v>1080000</v>
+        <v>2700000</v>
       </c>
       <c r="B28">
-        <v>25760840.699999999</v>
+        <v>2423310.9500000002</v>
       </c>
       <c r="C28">
-        <v>12975746.199999999</v>
+        <v>1364234.1</v>
       </c>
       <c r="D28">
-        <v>20098544.350000001</v>
+        <v>2219170.2999999998</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29">
-        <v>1120000</v>
+        <v>2800000</v>
       </c>
       <c r="B29">
-        <v>25520049.75</v>
+        <v>2236843.6</v>
       </c>
       <c r="C29">
-        <v>12981452</v>
+        <v>1315081.3999999999</v>
       </c>
       <c r="D29">
-        <v>20213931.649999999</v>
+        <v>2127354.25</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30">
-        <v>1160000</v>
+        <v>2900000</v>
       </c>
       <c r="B30">
-        <v>26055262.600000001</v>
+        <v>2235982.4500000002</v>
       </c>
       <c r="C30">
-        <v>13174044.5</v>
+        <v>1319610.6499999999</v>
       </c>
       <c r="D30">
-        <v>20531292.25</v>
+        <v>2118675.9</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31">
-        <v>1200000</v>
+        <v>3000000</v>
       </c>
       <c r="B31">
-        <v>25990273.350000001</v>
+        <v>2247601.25</v>
       </c>
       <c r="C31">
-        <v>13201579.449999999</v>
+        <v>1340089.45</v>
       </c>
       <c r="D31">
-        <v>20529016</v>
+        <v>2126855.4500000002</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>3100000</v>
+      </c>
+      <c r="B32">
+        <v>2248765.5499999998</v>
+      </c>
+      <c r="C32">
+        <v>1339324.3500000001</v>
+      </c>
+      <c r="D32">
+        <v>2129893.0499999998</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>3200000</v>
+      </c>
+      <c r="B33">
+        <v>2506534.7999999998</v>
+      </c>
+      <c r="C33">
+        <v>1402569.65</v>
+      </c>
+      <c r="D33">
+        <v>2298258.5</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>3300000</v>
+      </c>
+      <c r="B34">
+        <v>2278272.25</v>
+      </c>
+      <c r="C34">
+        <v>1349274.9</v>
+      </c>
+      <c r="D34">
+        <v>2206322.7999999998</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <v>3400000</v>
+      </c>
+      <c r="B35">
+        <v>2351233.15</v>
+      </c>
+      <c r="C35">
+        <v>1395239.25</v>
+      </c>
+      <c r="D35">
+        <v>2224627.1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>3500000</v>
+      </c>
+      <c r="B36">
+        <v>2327192.4500000002</v>
+      </c>
+      <c r="C36">
+        <v>1430820.5</v>
+      </c>
+      <c r="D36">
+        <v>2162826.35</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>3600000</v>
+      </c>
+      <c r="B37">
+        <v>2334283.35</v>
+      </c>
+      <c r="C37">
+        <v>1378926.05</v>
+      </c>
+      <c r="D37">
+        <v>2224406.9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>3700000</v>
+      </c>
+      <c r="B38">
+        <v>2477672.1</v>
+      </c>
+      <c r="C38">
+        <v>1453784.2</v>
+      </c>
+      <c r="D38">
+        <v>2311302.75</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>3800000</v>
+      </c>
+      <c r="B39">
+        <v>2355185.4</v>
+      </c>
+      <c r="C39">
+        <v>1399157.7</v>
+      </c>
+      <c r="D39">
+        <v>2183803.5499999998</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>3900000</v>
+      </c>
+      <c r="B40">
+        <v>2367498.65</v>
+      </c>
+      <c r="C40">
+        <v>1455847.9</v>
+      </c>
+      <c r="D40">
+        <v>2191922.2000000002</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>4000000</v>
+      </c>
+      <c r="B41">
+        <v>2398683.0499999998</v>
+      </c>
+      <c r="C41">
+        <v>1487554.55</v>
+      </c>
+      <c r="D41">
+        <v>2219953.4500000002</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42">
+        <v>4100000</v>
+      </c>
+      <c r="B42">
+        <v>2392995.7000000002</v>
+      </c>
+      <c r="C42">
+        <v>1405669.75</v>
+      </c>
+      <c r="D42">
+        <v>2188174.4</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43">
+        <v>4200000</v>
+      </c>
+      <c r="B43">
+        <v>2506931.2000000002</v>
+      </c>
+      <c r="C43">
+        <v>1441242.55</v>
+      </c>
+      <c r="D43">
+        <v>2222342.5499999998</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44">
+        <v>4300000</v>
+      </c>
+      <c r="B44">
+        <v>2506721.35</v>
+      </c>
+      <c r="C44">
+        <v>1424099.3</v>
+      </c>
+      <c r="D44">
+        <v>2244952</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <v>4400000</v>
+      </c>
+      <c r="B45">
+        <v>2441812.15</v>
+      </c>
+      <c r="C45">
+        <v>1512604.8</v>
+      </c>
+      <c r="D45">
+        <v>2255852.2999999998</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46">
+        <v>4500000</v>
+      </c>
+      <c r="B46">
+        <v>2444845.5499999998</v>
+      </c>
+      <c r="C46">
+        <v>1445342.95</v>
+      </c>
+      <c r="D46">
+        <v>2324724.75</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47">
+        <v>4600000</v>
+      </c>
+      <c r="B47">
+        <v>2448101.85</v>
+      </c>
+      <c r="C47">
+        <v>1449203.8</v>
+      </c>
+      <c r="D47">
+        <v>2262398.85</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48">
+        <v>4700000</v>
+      </c>
+      <c r="B48">
+        <v>2476419</v>
+      </c>
+      <c r="C48">
+        <v>1462577.3</v>
+      </c>
+      <c r="D48">
+        <v>2264053.25</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49">
+        <v>4800000</v>
+      </c>
+      <c r="B49">
+        <v>2478129</v>
+      </c>
+      <c r="C49">
+        <v>1461769.35</v>
+      </c>
+      <c r="D49">
+        <v>2261888.4</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50">
+        <v>4900000</v>
+      </c>
+      <c r="B50">
+        <v>2498015.2000000002</v>
+      </c>
+      <c r="C50">
+        <v>1486407.65</v>
+      </c>
+      <c r="D50">
+        <v>2282574.4500000002</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51">
+        <v>5000000</v>
+      </c>
+      <c r="B51">
+        <v>2525736.6</v>
+      </c>
+      <c r="C51">
+        <v>1472798.25</v>
+      </c>
+      <c r="D51">
+        <v>2282040.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor: axes in te diagram
</commit_message>
<xml_diff>
--- a/4a/bst_benchmark.xlsx
+++ b/4a/bst_benchmark.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\tr3sl9\2_sem\4a\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4893B824-3641-454F-BAED-7B4A483F13C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B21824F-22B1-45D9-9809-6B337A95352F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{ED679D53-E4ED-41AE-BC7A-34F45A594A49}"/>
   </bookViews>
@@ -632,7 +632,17 @@
             </a:r>
             <a:r>
               <a:rPr lang="en-US" baseline="0"/>
-              <a:t> benchmark</a:t>
+              <a:t> benchmark (</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:effectLst/>
+              </a:rPr>
+              <a:t>operations are performed with count of elements = 1000</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" baseline="0"/>
+              <a:t>)</a:t>
             </a:r>
             <a:endParaRPr lang="ru-RU"/>
           </a:p>
@@ -1745,8 +1755,67 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Count</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" baseline="0"/>
+                  <a:t> elements in tree at the time of operation</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="ru-RU"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
+        <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
@@ -1810,6 +1879,65 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>TIne</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" baseline="0"/>
+                  <a:t> (nanoseconds)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="ru-RU"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>

</xml_diff>